<commit_message>
Fill Key Skills v2 and work-experience tabs for all 19 roles
Wider mid/high gap (mid ~top 6, high ~top 14, tie groups kept whole within caps),
judgement moves recorded in the evidence file's Tier_Table.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017iQ6WGta978fv9oWoE415m
</commit_message>
<xml_diff>
--- a/key_skills_v2/fresh_grad_resumes_rebuild_ks2.xlsx
+++ b/key_skills_v2/fresh_grad_resumes_rebuild_ks2.xlsx
@@ -6348,8 +6348,21 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
-      <c r="C2" s="9" t="n"/>
-      <c r="D2" s="9" t="n"/>
+      <c r="C2" s="9" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: JavaScript, CSS, HTML
+\item Frameworks: REST APIs, React, Node.js
+\item Tools: Database Management (MySQL), Version Control (Git)
+\item Practices: Debugging, Software Testing, Backend Development, Frontend Development, API Integration, Performance Optimization, Responsive Web Design</t>
+        </is>
+      </c>
+      <c r="D2" s="9" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: JavaScript, CSS, HTML
+\item Frameworks: REST APIs, React
+\item Tools: Database Management, Version Control (Git)</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="10" t="n"/>
@@ -6358,8 +6371,22 @@
           <t>Back End Developer</t>
         </is>
       </c>
-      <c r="C3" s="11" t="n"/>
-      <c r="D3" s="11" t="n"/>
+      <c r="C3" s="11" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: SQL, JavaScript, CSS, HTML
+\item Frameworks: REST APIs
+\item Tools: Database Management (MySQL), Version Control (Git)
+\item Practices: Clean Code, Debugging, Troubleshooting, Backend Development, Code Review, Software Testing, Documentation, OOP</t>
+        </is>
+      </c>
+      <c r="D3" s="11" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: SQL, JavaScript
+\item Frameworks: REST APIs
+\item Tools: Database Management, Version Control (Git)
+\item Practices: Clean Code, Debugging, Troubleshooting</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="10" t="n"/>
@@ -6378,8 +6405,22 @@
           <t>Front End Developer</t>
         </is>
       </c>
-      <c r="C5" s="13" t="n"/>
-      <c r="D5" s="13" t="n"/>
+      <c r="C5" s="13" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: CSS, HTML, JavaScript
+\item Frameworks: React, Angular
+\item Tools: Version Control (Git)
+\item Practices: Frontend Development, Responsive Web Design, Performance Optimization, Software Testing, UI/UX Design, Clean Code, Web Development, Debugging</t>
+        </is>
+      </c>
+      <c r="D5" s="13" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: CSS, HTML, JavaScript
+\item Frameworks: React
+\item Tools: Version Control
+\item Practices: Frontend Development, Responsive Web Design</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="14" t="inlineStr">
@@ -6392,8 +6433,20 @@
           <t>Data Engineer</t>
         </is>
       </c>
-      <c r="C6" s="15" t="n"/>
-      <c r="D6" s="9" t="n"/>
+      <c r="C6" s="15" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: Python, SQL
+\item Tools: Database Management, Cloud Computing
+\item Practices: Data Pipelines, Data Quality, Big Data, Algorithms, Data Integration, ETL, Performance Optimization, Programming</t>
+        </is>
+      </c>
+      <c r="D6" s="9" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: Python, SQL
+\item Tools: Database Management, Cloud Computing
+\item Practices: Data Pipelines, Data Quality</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="10" t="n"/>
@@ -6405,7 +6458,7 @@
       <c r="C7" s="11" t="inlineStr">
         <is>
           <t>\item Languages \&amp; Queries: SQL, Python
-\item Tools: Power BI
+\item Tools: Power BI, Tableau
 \item Practices: Data Analysis, Dashboards, Data Quality, Data Collection, Reporting, Trend Analysis, Data Cleaning, Insight Generation, Statistics, Data Visualization</t>
         </is>
       </c>
@@ -6413,7 +6466,7 @@
         <is>
           <t>\item Languages \&amp; Queries: SQL
 \item Tools: Power BI
-\item Practices: Data Analysis, Dashboards, Data Quality, Data Collection, Reporting, Trend Analysis</t>
+\item Practices: Data Analysis, Dashboards, Data Quality, Data Collection, Reporting</t>
         </is>
       </c>
     </row>
@@ -6448,8 +6501,17 @@
           <t>Automation Test Engineer</t>
         </is>
       </c>
-      <c r="C10" s="9" t="n"/>
-      <c r="D10" s="9" t="n"/>
+      <c r="C10" s="9" t="inlineStr">
+        <is>
+          <t>\item Tools: Selenium, Jira, Version Control
+\item Practices: Defect Tracking \&amp; Bug Reporting, Test Case Design, Test Automation, Manual Testing, Agile / Scrum, Test Execution, Test Planning, Quality Assurance, Regression Testing, Requirements Gathering, Documentation, Mobile Testing, Test Reporting</t>
+        </is>
+      </c>
+      <c r="D10" s="9" t="inlineStr">
+        <is>
+          <t>\item Practices: Defect Tracking \&amp; Bug Reporting, Test Case Design, Test Automation, Manual Testing, Agile / Scrum, Test Execution</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="10" t="n"/>
@@ -6482,8 +6544,20 @@
           <t>DevOps Engineer</t>
         </is>
       </c>
-      <c r="C13" s="9" t="n"/>
-      <c r="D13" s="9" t="n"/>
+      <c r="C13" s="9" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: Python
+\item Tools: Cloud Computing (AWS, Azure), Terraform, Docker, Kubernetes, Linux
+\item Networking: Computer Networking
+\item Practices: Troubleshooting, Application Monitoring, Automation, Deployment, Scripting (Shell Scripting), CI/CD, Infrastructure as Code</t>
+        </is>
+      </c>
+      <c r="D13" s="9" t="inlineStr">
+        <is>
+          <t>\item Tools: Cloud Computing (AWS)
+\item Practices: Troubleshooting, Application Monitoring, Automation, Deployment, CI/CD</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="16" t="inlineStr">
@@ -6520,8 +6594,18 @@
           <t>UI/UX Designer</t>
         </is>
       </c>
-      <c r="C16" s="18" t="n"/>
-      <c r="D16" s="18" t="n"/>
+      <c r="C16" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Adobe Illustrator, Figma, Photoshop
+\item Practices: UI/UX Design, Brand Consistency, Responsive Web Design, Wireframing, Visual Design, Color Theory, Prototyping \&amp; Mockups, Requirements Gathering, Typography, Design Systems, Graphic Design, Web Development</t>
+        </is>
+      </c>
+      <c r="D16" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Adobe Illustrator, Figma, Photoshop
+\item Practices: UI/UX Design, Brand Consistency, Responsive Web Design, Wireframing, Visual Design</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="18" t="inlineStr">
@@ -6534,8 +6618,20 @@
           <t>BI / Reporting Developer</t>
         </is>
       </c>
-      <c r="C17" s="18" t="n"/>
-      <c r="D17" s="18" t="n"/>
+      <c r="C17" s="18" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: SQL
+\item Tools: MS Office (MS Excel, Pivot Tables), Power BI (DAX), Database Management
+\item Practices: Dashboards, Reporting, Data Modeling, Documentation, Data Validation, Data Warehousing, Dimensional Modeling, Requirements Gathering, Data Cleaning</t>
+        </is>
+      </c>
+      <c r="D17" s="18" t="inlineStr">
+        <is>
+          <t>\item Languages \&amp; Queries: SQL
+\item Tools: MS Office (MS Excel), Power BI
+\item Practices: Dashboards, Reporting, Documentation</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="18" t="inlineStr">
@@ -6548,8 +6644,19 @@
           <t>Network Engineer</t>
         </is>
       </c>
-      <c r="C18" s="18" t="n"/>
-      <c r="D18" s="18" t="n"/>
+      <c r="C18" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Linux, Ticketing / ITSM Tools, Windows
+\item Networking: Computer Networking, Network Monitoring, Network Troubleshooting, Routers \&amp; Switches, Firewalls, LAN / WAN, Network Security
+\item Practices: Troubleshooting, Documentation, Technical Support, Equipment Installation, Incident Management</t>
+        </is>
+      </c>
+      <c r="D18" s="18" t="inlineStr">
+        <is>
+          <t>\item Networking: Computer Networking, Network Monitoring, Network Troubleshooting, Routers \&amp; Switches
+\item Practices: Troubleshooting, Documentation, Technical Support</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="18" t="inlineStr">
@@ -6562,8 +6669,16 @@
           <t>Field Technician</t>
         </is>
       </c>
-      <c r="C19" s="18" t="n"/>
-      <c r="D19" s="18" t="n"/>
+      <c r="C19" s="18" t="inlineStr">
+        <is>
+          <t>\item Practices: Troubleshooting, Equipment Servicing \&amp; Repair, Equipment Installation, Preventive Maintenance, Technical Support, Reporting, Documentation, Electrical Systems, Quality Control / Inspection, Record Keeping, Customer Query Handling, User Training, Commissioning, Workplace Safety, Mechanical Systems, Electronics</t>
+        </is>
+      </c>
+      <c r="D19" s="18" t="inlineStr">
+        <is>
+          <t>\item Practices: Troubleshooting, Equipment Servicing \&amp; Repair, Equipment Installation, Preventive Maintenance, Technical Support, Reporting</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="18" t="inlineStr">
@@ -6571,8 +6686,20 @@
           <t>IT Infra / Support Engineer</t>
         </is>
       </c>
-      <c r="C20" s="18" t="n"/>
-      <c r="D20" s="18" t="n"/>
+      <c r="C20" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Windows, MS Office, Ticketing / ITSM Tools, Operating Systems
+\item Networking: Computer Networking, Network Troubleshooting
+\item Practices: Troubleshooting, Documentation, Desktop Support, Technical Support, IT Support, Hardware Troubleshooting \&amp; Repair, Software Installation \&amp; Patching, Printer \&amp; Peripheral Support, IT Asset Management, Remote Support</t>
+        </is>
+      </c>
+      <c r="D20" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Windows
+\item Networking: Computer Networking, Network Troubleshooting
+\item Practices: Troubleshooting, Documentation, Desktop Support, Technical Support, IT Support</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="18" t="inlineStr">
@@ -6585,8 +6712,18 @@
           <t>Information Security / SOC Analyst</t>
         </is>
       </c>
-      <c r="C21" s="18" t="n"/>
-      <c r="D21" s="18" t="n"/>
+      <c r="C21" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Linux
+\item Networking: Computer Networking
+\item Practices: Documentation, Vulnerability Assessment, Incident Response, Security Monitoring, Alert Triage, Escalation Handling, Information Security, SIEM, EDR, Cloud Security, Compliance, Log Analysis, Reporting, Threat Intelligence</t>
+        </is>
+      </c>
+      <c r="D21" s="18" t="inlineStr">
+        <is>
+          <t>\item Practices: Documentation, Vulnerability Assessment, Incident Response, Security Monitoring, Alert Triage, SIEM</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="18" t="inlineStr">
@@ -6599,8 +6736,19 @@
           <t>ERP Consultant</t>
         </is>
       </c>
-      <c r="C22" s="18" t="n"/>
-      <c r="D22" s="18" t="n"/>
+      <c r="C22" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: ERP Systems (SAP), MS Office (MS Excel)
+\item Practices: Documentation, Requirements Gathering, Software Testing (UAT), User Training, ERP Implementation \&amp; Support, SAP / ERP Configuration, Troubleshooting, Technical Support, Process Mapping, Reporting, ERP Integration, Master Data Management
+\item Languages: English</t>
+        </is>
+      </c>
+      <c r="D22" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: ERP Systems
+\item Practices: Documentation, Requirements Gathering, Software Testing, User Training, ERP Implementation \&amp; Support</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="B23" s="18" t="inlineStr">
@@ -6608,8 +6756,18 @@
           <t>SAP Technical Consultant</t>
         </is>
       </c>
-      <c r="C23" s="18" t="n"/>
-      <c r="D23" s="18" t="n"/>
+      <c r="C23" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: SAP (SAP ABAP, SAP S/4HANA, SAP MM), Database Management
+\item Practices: Documentation, Software Testing, Troubleshooting, Reporting, Requirements Gathering, SAP / ERP Configuration, Debugging, Software Architecture, Technical Support, ERP Implementation \&amp; Support</t>
+        </is>
+      </c>
+      <c r="D23" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: SAP (SAP ABAP, SAP S/4HANA)
+\item Practices: Documentation, Software Testing, Troubleshooting, SAP / ERP Configuration</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="18" t="inlineStr">
@@ -6629,7 +6787,7 @@
       </c>
       <c r="D24" s="18" t="inlineStr">
         <is>
-          <t>\item Practices: Inventory Management, Inbound / Receiving, Compliance, Record Keeping, Reporting, Outbound / Dispatch, Discrepancy \&amp; Damage Reporting, Logistics Operations, Warehouse Operations, Operations Management</t>
+          <t>\item Practices: Inventory Management, Inbound / Receiving, Compliance, Record Keeping, Reporting, Outbound / Dispatch</t>
         </is>
       </c>
     </row>
@@ -6644,8 +6802,19 @@
           <t>HR / Talent Acquisition Specialist</t>
         </is>
       </c>
-      <c r="C25" s="18" t="n"/>
-      <c r="D25" s="18" t="n"/>
+      <c r="C25" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Job Portals (Naukri / LinkedIn)
+\item Practices: Sourcing, Recruitment (End-to-end), Candidate Screening, Interview Coordination, Recruitment Trackers \&amp; MIS, Bulk / Volume Hiring, Interviewing, Talent Pipeline, Onboarding, Non-IT Recruitment, Requirements Gathering, Offer \&amp; Salary Negotiation, Reporting, Technical / Engineering Recruitment
+\item Languages: English</t>
+        </is>
+      </c>
+      <c r="D25" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Job Portals (Naukri / LinkedIn)
+\item Practices: Sourcing, Recruitment (End-to-end), Candidate Screening, Interview Coordination, Recruitment Trackers \&amp; MIS</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="B26" s="18" t="inlineStr">
@@ -6653,8 +6822,18 @@
           <t>Finance and Accounts Executive</t>
         </is>
       </c>
-      <c r="C26" s="18" t="n"/>
-      <c r="D26" s="18" t="n"/>
+      <c r="C26" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: MS Office (MS Excel), ERP Systems, Tally
+\item Practices: Invoice Processing \&amp; Billing, Accounting, Account Reconciliation, Record Keeping, Accounts Payable, Accounts Receivable, Month-end Closing, Reporting, Vendor Management, Audit Support, Compliance, Documentation, Bookkeeping</t>
+        </is>
+      </c>
+      <c r="D26" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: MS Office (MS Excel), Tally
+\item Practices: Invoice Processing \&amp; Billing, Accounting, Account Reconciliation, Record Keeping</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="18" t="inlineStr">
@@ -6667,8 +6846,20 @@
           <t>Customer Support Associate</t>
         </is>
       </c>
-      <c r="C27" s="18" t="n"/>
-      <c r="D27" s="18" t="n"/>
+      <c r="C27" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Basic Computer Skills, Ticketing / ITSM Tools
+\item Practices: Customer Query Handling, Inbound / Outbound Call Handling, Product Knowledge, Escalation Handling, Record Keeping, SOP Compliance, Chat \&amp; Email Support, Call Center Metrics (AHT / CSAT), Data Entry, Troubleshooting, Customer Relationship Management
+\item Languages: English</t>
+        </is>
+      </c>
+      <c r="D27" s="18" t="inlineStr">
+        <is>
+          <t>\item Tools: Basic Computer Skills
+\item Practices: Customer Query Handling, Inbound / Outbound Call Handling, Product Knowledge, Escalation Handling, Record Keeping, SOP Compliance
+\item Languages: English</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -6768,6 +6959,106 @@
           <t>Full Stack Developer</t>
         </is>
       </c>
+      <c r="B2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built frontend development features for a partner-integration portal with React, JavaScript, HTML and CSS, using responsive web design.
+\item Developed backend development modules and REST APIs in Node.js for service-partner data.
+\item Led API integration with OEM and third-party partner tools, cutting manual partner updates by about 30\%.
+\item Designed MySQL tables and handled database management for partner records.
+\item Used Git for version control and carried out debugging, software testing and performance optimization before each release.</t>
+        </is>
+      </c>
+      <c r="C2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built responsive web design layouts and frontend development screens in React, JavaScript, HTML and CSS for a social-media data app.
+\item Developed Node.js backend development services and REST APIs to process incoming social-media data.
+\item Handled database management in MySQL, designing tables for large post and profile datasets.
+\item Added new data sources through API integration with third-party social-media APIs.
+\item Led debugging, software testing and performance optimization with Git version control, improving page load time by about 25\%.</t>
+        </is>
+      </c>
+      <c r="D2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Maintained the central database, owning database management and MySQL schema changes.
+\item Developed backend development services and REST APIs in Node.js on top of the central database.
+\item Created frontend development pages in React, JavaScript, HTML and CSS with responsive web design.
+\item Delivered API integration with third-party tools used by business teams.
+\item Improved page speed through performance optimization, debugging and software testing tracked in Git version control, reducing response time by about 20\%.</t>
+        </is>
+      </c>
+      <c r="E2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built a support portal through frontend development in React, JavaScript, HTML and CSS using responsive web design.
+\item Developed REST APIs and backend development services in Node.js for first-level issue triaging.
+\item Handled database management for stored support requests in MySQL.
+\item Led API integration with third-party tools so support requests flowed between systems.
+\item Fixed issues through debugging and software testing, applied performance optimization, and kept code in Git version control.</t>
+        </is>
+      </c>
+      <c r="F2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built responsive web design components and frontend development features in React, JavaScript, HTML and CSS for platform solutions.
+\item Developed backend development services and REST APIs in Node.js.
+\item Owned database management for the platform in MySQL.
+\item Delivered API integration with third-party services, reducing manual work by about 30\%.
+\item Carried out debugging, software testing and performance optimization, with all changes tracked in Git version control.</t>
+        </is>
+      </c>
+      <c r="G2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building React components with JavaScript for a partner-integration portal.
+\item Supported page updates by writing HTML and CSS.
+\item Helped connect screens to REST APIs for service-partner data.
+\item Supported database management tasks such as updating tables.
+\item Used Git for version control on shared code.</t>
+        </is>
+      </c>
+      <c r="H2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building React screens in JavaScript for a social-media data app.
+\item Wrote HTML and CSS for new pages and small fixes.
+\item Helped call REST APIs that returned social-media data.
+\item Supported database management by maintaining tables for stored data.
+\item Committed code changes to Git for version control.</t>
+        </is>
+      </c>
+      <c r="I2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Supported database management for the central database, updating tables.
+\item Assisted in building React components with JavaScript.
+\item Wrote HTML and CSS for internal pages.
+\item Helped consume REST APIs that read from the central database.
+\item Used Git for version control on every change.</t>
+        </is>
+      </c>
+      <c r="J2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building React screens with JavaScript for a support portal.
+\item Wrote HTML and CSS for portal pages.
+\item Helped wire portal forms to REST APIs.
+\item Supported database management for stored support requests.
+\item Used Git for version control during issue triaging work.</t>
+        </is>
+      </c>
+      <c r="K2" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in developing React components in JavaScript for platform solutions.
+\item Wrote HTML and CSS for platform pages.
+\item Helped build and consume REST APIs.
+\item Supported database management tasks for the platform.
+\item Used Git for version control and code updates.</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="30" t="inlineStr">
@@ -6775,6 +7066,106 @@
           <t>Back End Developer</t>
         </is>
       </c>
+      <c r="B3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built backend development services and REST APIs for application maintenance work using OOP principles.
+\item Designed MySQL schemas, wrote SQL queries and handled database management for product and order data.
+\item Wrote clean code with documentation and took part in code reviews, using Git version control.
+\item Led software testing, debugging and troubleshooting of services, cutting defect fix time by about 25\%.
+\item Built supporting screens in JavaScript, HTML and CSS for the maintained applications.</t>
+        </is>
+      </c>
+      <c r="C3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built scalable REST APIs through backend development, applying OOP design.
+\item Owned database management in MySQL, writing efficient SQL queries.
+\item Led code reviews and wrote clean code with clear documentation, tracked in Git version control.
+\item Improved API reliability by about 20\% through software testing, debugging and troubleshooting.
+\item Built simple admin pages with JavaScript, HTML and CSS.</t>
+        </is>
+      </c>
+      <c r="D3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Built backend development modules and REST APIs for internal tools using OOP.
+\item Wrote SQL queries in MySQL and handled database management for tool data.
+\item Created tool front ends in JavaScript, HTML and CSS.
+\item Wrote clean code with documentation, kept in Git version control and checked in code reviews.
+\item Led software testing, debugging and troubleshooting, reducing repeat issues by about 30\%.</t>
+        </is>
+      </c>
+      <c r="E3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Developed backend development services and REST APIs for a data-driven business application with OOP.
+\item Wrote SQL queries against MySQL for application work and handled database management.
+\item Led troubleshooting and debugging of data issues, plus software testing of each change.
+\item Wrote clean code and documentation, with Git version control and peer code reviews.
+\item Built user screens in JavaScript, HTML and CSS, cutting page errors by about 20\%.</t>
+        </is>
+      </c>
+      <c r="F3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Resolved technical issues reported by QA and end-users through troubleshooting and debugging, cutting open issues by about 30\%.
+\item Built backend development fixes and new REST APIs using OOP.
+\item Handled database management tasks in MySQL and wrote SQL queries for fixes.
+\item Wrote clean code and documentation, using Git version control and code reviews.
+\item Ran software testing on fixes and updated JavaScript, HTML and CSS screens.</t>
+        </is>
+      </c>
+      <c r="G3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building REST APIs during application maintenance.
+\item Wrote basic SQL queries and supported database management tasks.
+\item Helped with debugging and troubleshooting of reported issues.
+\item Wrote clean code in JavaScript for small features.
+\item Used Git for version control.</t>
+        </is>
+      </c>
+      <c r="H3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building REST APIs for the API platform.
+\item Supported database management with simple SQL queries.
+\item Helped with debugging and troubleshooting of API errors.
+\item Followed clean code practices in JavaScript.
+\item Used Git version control for all changes.</t>
+        </is>
+      </c>
+      <c r="I3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Assisted in building REST APIs for internal tools.
+\item Wrote SQL queries and supported database management.
+\item Helped with debugging and troubleshooting tool errors.
+\item Wrote clean code in JavaScript.
+\item Tracked changes with Git version control.</t>
+        </is>
+      </c>
+      <c r="J3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Supported database management and wrote SQL queries for a data-driven business application.
+\item Assisted in building REST APIs.
+\item Helped with troubleshooting and debugging of data issues.
+\item Wrote clean code in JavaScript for screens.
+\item Used Git for version control.</t>
+        </is>
+      </c>
+      <c r="K3" s="30" t="inlineStr">
+        <is>
+          <t>Software Developer I
+\item Helped resolve issues reported by QA and end-users through debugging and troubleshooting.
+\item Assisted in updating REST APIs.
+\item Wrote SQL queries and supported database management.
+\item Wrote clean code in JavaScript for fixes.
+\item Used Git for version control.</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="30" t="inlineStr">
@@ -6782,11 +7173,211 @@
           <t>Front End Developer</t>
         </is>
       </c>
+      <c r="B4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Built frontend development features for software solutions in React and Angular, using JavaScript, HTML and CSS.
+\item Delivered responsive web design layouts and turned UI/UX design ideas into working screens.
+\item Wrote clean code and reusable components, using Git for version control.
+\item Led performance optimization through lazy loading and code splitting, cutting page load time by about 30\%.
+\item Handled debugging and software testing of interfaces before each web development release.</t>
+        </is>
+      </c>
+      <c r="C4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Led web development of the company website from concept to completion, from the home page to site layout.
+\item Built frontend development pages in React and Angular with JavaScript, HTML and CSS, using responsive web design.
+\item Applied UI/UX design ideas so the site stayed functional and appealing.
+\item Wrote clean code tracked in Git version control, and handled debugging and software testing.
+\item Improved site speed through performance optimization, reducing load time by about 25\%.</t>
+        </is>
+      </c>
+      <c r="D4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Built frontend development screens that render correctly on multiple platforms, using React, Angular, JavaScript, HTML and CSS.
+\item Delivered responsive web design across devices and checked the technical feasibility of UI/UX design.
+\item Led software testing of user interfaces on multiple platforms, plus debugging of rendering issues.
+\item Wrote clean code with Git version control for each web development change.
+\item Improved rendering speed by about 20\% through performance optimization.</t>
+        </is>
+      </c>
+      <c r="E4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Built new user-facing features through frontend development in React and Angular with JavaScript, HTML and CSS.
+\item Applied responsive web design and UI/UX design input to each feature.
+\item Wrote clean code and reusable components, using Git version control.
+\item Handled debugging and software testing of new features as part of web development.
+\item Led performance optimization of key screens, cutting load time by about 30\%.</t>
+        </is>
+      </c>
+      <c r="F4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Led web development work on web application products, building frontend development features in React and Angular.
+\item Wrote JavaScript, HTML and CSS for responsive web design layouts.
+\item Shaped UI/UX design across product screens and turned it into clean code.
+\item Used Git version control and carried out debugging and software testing.
+\item Improved product speed by about 20\% through performance optimization.</t>
+        </is>
+      </c>
+      <c r="G4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Assisted in frontend development of user interfaces for software solutions.
+\item Wrote HTML and CSS for new screens.
+\item Supported React components written in JavaScript.
+\item Helped apply responsive web design across devices.
+\item Used version control tools to manage code changes.</t>
+        </is>
+      </c>
+      <c r="H4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Assisted in frontend development of the company website.
+\item Wrote HTML and CSS for the home page and site layout.
+\item Helped build React components with JavaScript.
+\item Supported responsive web design so pages worked on phones.
+\item Committed changes through version control tools.</t>
+        </is>
+      </c>
+      <c r="I4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Supported frontend development of screens used on multiple platforms.
+\item Wrote HTML and CSS for layouts.
+\item Helped build React components in JavaScript.
+\item Assisted with responsive web design across devices.
+\item Tracked code changes in version control.</t>
+        </is>
+      </c>
+      <c r="J4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Assisted in frontend development of new user-facing features.
+\item Wrote HTML, CSS and JavaScript for feature screens.
+\item Helped build React components.
+\item Supported responsive web design for each feature.
+\item Used version control tools for all changes.</t>
+        </is>
+      </c>
+      <c r="K4" s="30" t="inlineStr">
+        <is>
+          <t>Front End Developer I
+\item Supported frontend development for web application products.
+\item Wrote HTML and CSS for product pages.
+\item Assisted in building React components with JavaScript.
+\item Helped make layouts follow responsive web design.
+\item Used version control to track updates.</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="30" t="inlineStr">
         <is>
           <t>Data Engineer</t>
+        </is>
+      </c>
+      <c r="B5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Built and maintained production data pipelines in Python and SQL.
+\item Led ETL work and data integration from databases, files and APIs into the cloud.
+\item Improved pipeline speed by about 30\% through performance optimization of SQL queries.
+\item Added data quality checks to protect data integrity in big data jobs.
+\item Wrote algorithms in Python programming to handle large production data volumes.</t>
+        </is>
+      </c>
+      <c r="C5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Built data pipelines that bring together data from various client systems.
+\item Led data integration and ETL from client databases into cloud storage.
+\item Wrote Python programming logic, SQL and algorithms to match client records.
+\item Added data quality checks across big data loads from client systems.
+\item Improved load times by about 25\% through performance optimization.</t>
+        </is>
+      </c>
+      <c r="D5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Built data pipelines that feed large datasets into AI projects.
+\item Led ETL and data integration from databases and cloud sources using Python and SQL.
+\item Applied data quality checks to keep model input data accurate.
+\item Built big data jobs and algorithms for large-scale data handling.
+\item Improved job run time by about 20\% through performance optimization and better programming practices.</t>
+        </is>
+      </c>
+      <c r="E5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Built data pipelines for a high-visibility project in Python and SQL.
+\item Led ETL and data integration across databases, files and APIs.
+\item Designed big data jobs on cloud platforms, applying programming and algorithms skills.
+\item Improved query speed by about 30\% through performance optimization.
+\item Added data quality checks that kept project data consistent.</t>
+        </is>
+      </c>
+      <c r="F5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Built scalable data pipelines that support data-driven business solutions.
+\item Led data integration and ETL from source databases into cloud platforms.
+\item Wrote Python and SQL programming logic, including algorithms for large data volumes.
+\item Ran big data workloads and added data quality checks.
+\item Improved pipeline speed by about 25\% through performance optimization.</t>
+        </is>
+      </c>
+      <c r="G5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Assisted in keeping production data pipelines running.
+\item Wrote basic Python and SQL code for pipeline tasks.
+\item Supported routine work on relational databases.
+\item Helped run data quality checks for data integrity.
+\item Gained exposure to cloud platforms used by the team.</t>
+        </is>
+      </c>
+      <c r="H5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Assisted in maintaining data pipelines that bring together client-system data.
+\item Wrote SQL queries and Python code to load client records.
+\item Supported work on client databases.
+\item Helped run data quality checks on incoming data.
+\item Learned cloud platforms used for storage.</t>
+        </is>
+      </c>
+      <c r="I5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Supported data pipelines that feed large datasets into AI projects.
+\item Wrote Python and SQL code for pipeline steps.
+\item Helped maintain project databases.
+\item Assisted with data quality checks on project data.
+\item Worked with cloud tools under senior guidance.</t>
+        </is>
+      </c>
+      <c r="J5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Assisted in building data pipelines for a high-visibility project.
+\item Wrote SQL and Python code for pipeline steps.
+\item Supported database tasks for the project.
+\item Helped run data quality checks.
+\item Gained exposure to cloud platforms.</t>
+        </is>
+      </c>
+      <c r="K5" s="30" t="inlineStr">
+        <is>
+          <t>Data Engineer I
+\item Supported data pipelines for data-driven business solutions.
+\item Wrote basic Python and SQL code.
+\item Helped maintain source databases.
+\item Assisted with data quality checks and fixes.
+\item Learned to use cloud platforms for data storage.</t>
         </is>
       </c>
     </row>
@@ -6801,7 +7392,7 @@
           <t>Data Analyst I
 \item Built SQL queries to collect and analyze security operations data from multiple sources.
 \item Cleaned and standardized raw security data logs in Python to improve data quality and integrity.
-\item Designed real-time Power BI dashboards and data visualizations for the operations team.
+\item Designed real-time Power BI and Tableau dashboards and data visualizations for the operations team.
 \item Applied statistical analysis to identify emerging security trends and generate actionable insights.
 \item Compiled security operational reports, cutting weekly report preparation time by about 20\%.</t>
         </is>
@@ -6811,27 +7402,27 @@
           <t>Data Analyst I
 \item Built SQL queries to collect and analyze large, complex financial datasets from multiple sources.
 \item Cleaned and restructured raw financial data in Python, improving data quality across reports.
-\item Developed Power BI dashboards and data visualizations to monitor financial data.
+\item Developed Power BI and Tableau dashboards and data visualizations to monitor financial data.
 \item Used statistical techniques to identify trends, patterns and anomalies, turning them into actionable insights.
-\item Prepared detailed recurring reports from the analysis, cutting turnaround time by about 15\%.</t>
+\item Prepared detailed recurring reports from the work, cutting turnaround time by about 15\%.</t>
         </is>
       </c>
       <c r="D6" s="30" t="inlineStr">
         <is>
           <t>Data Analyst I
-\item Collected and analyzed portfolio and product data using SQL for deep-dive analysis.
-\item Cleaned and preprocessed raw datasets in Python, improving data quality before analysis.
-\item Built Power BI dashboards and data visualizations to monitor portfolio performance.
-\item Applied statistical analysis to identify trends and patterns and generate actionable insights on products.
-\item Led regular reporting across products, reducing ad-hoc report requests by about 20\%.</t>
+\item Collected and analyzed portfolio and product data using SQL for deep-dive work.
+\item Cleaned and preprocessed raw datasets in Python, improving data quality before use.
+\item Built Power BI and Tableau dashboards and data visualizations to monitor portfolio performance.
+\item Applied statistical techniques to identify trends and patterns and generate actionable insights on products.
+\item Led regular reporting across products, reducing one-off report requests by about 20\%.</t>
         </is>
       </c>
       <c r="E6" s="30" t="inlineStr">
         <is>
           <t>Data Analyst I
-\item Collected large datasets from diverse sources and wrote SQL queries for ad-hoc analysis for leadership.
+\item Collected large datasets from diverse sources and wrote SQL queries so leadership could see them analyzed quickly.
 \item Cleaned raw data in Python and improved data quality by building checks that flag data issues.
-\item Built intuitive Power BI dashboards and data visualizations for leadership reviews.
+\item Built intuitive Power BI and Tableau dashboards and data visualizations for leadership reviews.
 \item Applied statistical modelling to spot trends and transform raw data into actionable insights.
 \item Delivered enterprise reports for leadership, improving report turnaround by about 25\%.</t>
         </is>
@@ -6841,7 +7432,7 @@
           <t>Data Analyst I
 \item Collected and organized business data from various sources and analyzed it with SQL.
 \item Cleaned datasets in Python and set up data quality checks to catch inconsistencies.
-\item Built Power BI dashboards and data visualizations for business teams.
+\item Built Power BI and Tableau dashboards and data visualizations for business teams.
 \item Used statistics to identify trends and patterns and share actionable insights with business teams.
 \item Produced weekly reports for business teams, cutting manual report preparation by about 30\%.</t>
         </is>
@@ -6850,10 +7441,10 @@
         <is>
           <t>Data Analyst I
 \item Assisted in collecting security operations data from multiple sources.
-\item Supported data analysis by writing basic SQL queries to retrieve and analyze data.
+\item Supported data analysis by writing basic SQL queries to retrieve data.
 \item Helped maintain data quality through routine accuracy and consistency checks.
 \item Supported the team in maintaining Power BI dashboards for security operations.
-\item Helped compile security operational reports and flagged emerging trends for review.</t>
+\item Helped compile security operational reports for review.</t>
         </is>
       </c>
       <c r="H6" s="30" t="inlineStr">
@@ -6861,29 +7452,29 @@
           <t>Data Analyst I
 \item Assisted in collecting and organizing financial data from multiple sources.
 \item Wrote basic SQL queries to retrieve data and supported data analysis of financial datasets.
-\item Helped ensure data quality by checking reports for accuracy and consistency.
+\item Helped ensure data quality by checking figures for accuracy and consistency.
 \item Supported updates to Power BI dashboards used to monitor financial data.
-\item Helped prepare detailed reports and identify trends and patterns in financial datasets.</t>
+\item Helped prepare detailed monthly reports.</t>
         </is>
       </c>
       <c r="I6" s="30" t="inlineStr">
         <is>
           <t>Data Analyst I
-\item Assisted in collecting portfolio and product data for team analysis.
-\item Wrote basic SQL queries to retrieve data and supported deep-dive data analysis across products.
+\item Assisted in collecting portfolio and product data for the team.
+\item Wrote basic SQL queries to retrieve data and supported data analysis across products.
 \item Helped maintain data quality by flagging inconsistencies and quality issues.
 \item Supported maintenance of Power BI dashboards on portfolio performance.
-\item Helped prepare regular reports and identify trends in product data.</t>
+\item Helped prepare regular reports on product data.</t>
         </is>
       </c>
       <c r="J6" s="30" t="inlineStr">
         <is>
           <t>Data Analyst I
 \item Assisted in collecting large datasets from diverse sources.
-\item Wrote basic SQL queries to support ad-hoc data analysis for leadership.
+\item Wrote basic SQL queries to support data analysis for leadership.
 \item Helped improve data quality by logging and resolving data issues.
 \item Supported the build of Power BI dashboards for leadership reviews.
-\item Helped prepare recurring reports and highlighted key trends for senior analysts.</t>
+\item Helped prepare recurring reports for senior analysts.</t>
         </is>
       </c>
       <c r="K6" s="30" t="inlineStr">
@@ -6893,7 +7484,7 @@
 \item Wrote basic SQL queries and supported routine data analysis for business teams.
 \item Helped ensure data quality by following company processes for data accuracy.
 \item Supported creation of Power BI dashboards for business teams.
-\item Helped prepare basic reports and identify basic trends and patterns.</t>
+\item Helped prepare basic weekly reports.</t>
         </is>
       </c>
     </row>
@@ -6903,6 +7494,106 @@
           <t>Automation Test Engineer</t>
         </is>
       </c>
+      <c r="B7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Led test planning and test case design from business requirements as part of the quality assurance process for web applications.
+\item Built test automation scripts in Selenium and ran manual testing for new features.
+\item Logged defects in Jira with clear steps and drove bug reports to closure.
+\item Ran regression testing and test execution each sprint in an Agile / Scrum team, cutting escaped defects by about 25\%.
+\item Wrote test reporting and documentation kept under version control, and covered mobile testing of the web screens.</t>
+        </is>
+      </c>
+      <c r="C7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Led test planning and test case design for warehouse data loads, based on data requirements.
+\item Built Selenium test automation for the reporting front end and ran manual testing of data checks.
+\item Ran test execution and regression testing on each release in an Agile / Scrum team.
+\item Logged defects in Jira and wrote test reporting and documentation stored in version control.
+\item Improved quality assurance coverage by about 30\% and added mobile testing for the reporting app.</t>
+        </is>
+      </c>
+      <c r="D7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Led test planning and test case design for client web and mobile apps across real estate, e-commerce and fintech.
+\item Built Selenium test automation and ran manual testing and mobile testing across a range of devices.
+\item Ran regression testing and test execution every sprint under Agile / Scrum.
+\item Tracked defects in Jira and clarified requirements with client teams.
+\item Produced test reporting and documentation under version control, raising quality assurance pass rates by about 20\%.</t>
+        </is>
+      </c>
+      <c r="E7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Led test planning and test case design for game builds as part of the quality assurance process.
+\item Ran manual testing and mobile testing of games across low-end and high-end devices.
+\item Built Selenium test automation for the game's web portal.
+\item Logged bugs in Jira and ran regression testing on previously fixed defects, cutting reopened bugs by about 30\%.
+\item Ran test execution against requirements in Agile / Scrum sprints, with test reporting and documentation kept in version control.</t>
+        </is>
+      </c>
+      <c r="F7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Led test planning and test case design for web and AI applications from product requirements.
+\item Built test automation with Selenium and ran manual testing of new features.
+\item Ran test execution, regression testing and mobile testing in an Agile / Scrum team.
+\item Logged defects in Jira and wrote test reporting for each sprint.
+\item Kept documentation in version control, improving quality assurance turnaround by about 20\%.</t>
+        </is>
+      </c>
+      <c r="G7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Assisted in writing test cases for web applications and APIs.
+\item Performed manual testing of new features.
+\item Supported test execution and logged defects with clear steps.
+\item Helped maintain basic automation scripts.
+\item Took part in Agile / Scrum stand-ups and sprint reviews.</t>
+        </is>
+      </c>
+      <c r="H7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Assisted in writing test cases for warehouse data loads.
+\item Performed manual testing of data checks.
+\item Supported test execution and logged defects.
+\item Helped run simple automation scripts.
+\item Took part in Agile / Scrum ceremonies.</t>
+        </is>
+      </c>
+      <c r="I7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Assisted in writing test cases for client web apps.
+\item Performed manual testing of new screens.
+\item Supported test execution and logged bugs with screenshots.
+\item Helped build basic automation scripts.
+\item Joined Agile / Scrum sprint meetings.</t>
+        </is>
+      </c>
+      <c r="J7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Assisted in writing test cases for game builds.
+\item Performed manual testing of game features.
+\item Supported test execution and logged bugs with reproduction steps.
+\item Helped with basic test automation of repeat checks.
+\item Took part in Agile / Scrum stand-ups.</t>
+        </is>
+      </c>
+      <c r="K7" s="30" t="inlineStr">
+        <is>
+          <t>QA Engineer I
+\item Assisted in writing test cases for web and AI applications.
+\item Performed manual testing of new features.
+\item Supported test execution and logged defects.
+\item Helped run test automation with modern tools.
+\item Took part in Agile / Scrum sprint meetings.</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="30" t="inlineStr">
@@ -6910,6 +7601,106 @@
           <t>DevOps Engineer</t>
         </is>
       </c>
+      <c r="B8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Built and ran AWS and Azure cloud environments for global clients using infrastructure as code in Terraform.
+\item Led CI/CD pipelines that automated build and deployment for client applications.
+\item Packaged services with Docker and ran them on Kubernetes clusters.
+\item Wrote Python and shell scripting for routine tasks on Linux servers.
+\item Improved uptime by about 20\% through application monitoring, troubleshooting and fixing networking issues.</t>
+        </is>
+      </c>
+      <c r="C8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Managed AWS cloud services and Azure resources for distributed systems.
+\item Built CI/CD pipelines for automated deployment of Docker images to Kubernetes.
+\item Wrote Terraform for infrastructure as code, plus Python and shell scripting for routine tasks.
+\item Led troubleshooting across Linux hosts, networking and applications.
+\item Set up application monitoring and alerts, cutting time to detect issues by about 25\%.</t>
+        </is>
+      </c>
+      <c r="D8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Led migration of client workloads from AWS and Azure to a new cloud platform.
+\item Wrote Terraform as infrastructure as code for the target cloud setup.
+\item Built CI/CD pipelines and automated deployment of Docker images on Kubernetes.
+\item Wrote Python and shell scripting for migration steps on Linux servers.
+\item Improved post-migration stability by about 20\% through application monitoring, troubleshooting and networking checks.</t>
+        </is>
+      </c>
+      <c r="E8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Built cloud infrastructure on AWS and Azure for cloud native products.
+\item Led CI/CD pipelines with automated build and deployment.
+\item Ran product services in Docker on Kubernetes, defined through Terraform infrastructure as code.
+\item Wrote Python and shell scripting for automation on Linux.
+\item Improved release reliability by about 30\% with application monitoring and troubleshooting, including networking issues.</t>
+        </is>
+      </c>
+      <c r="F8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Designed secure, high-availability cloud infrastructure on AWS and Azure using Terraform infrastructure as code.
+\item Built CI/CD pipelines for automated deployment of Docker images to Kubernetes.
+\item Wrote Python and shell scripting to automate Linux server tasks.
+\item Led troubleshooting of networking and application issues during outages.
+\item Improved availability by about 20\% through application monitoring and alerting.</t>
+        </is>
+      </c>
+      <c r="G8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Assisted in maintaining AWS cloud environments for global clients.
+\item Supported CI/CD pipelines for application deployment.
+\item Helped monitor systems, respond to alerts and follow runbooks.
+\item Assisted in troubleshooting issues raised by clients.
+\item Supported automation of routine tasks.</t>
+        </is>
+      </c>
+      <c r="H8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Assisted in maintaining AWS cloud services for distributed systems.
+\item Supported deployment of applications through CI/CD pipelines.
+\item Helped monitor system health.
+\item Assisted in troubleshooting service issues.
+\item Supported automation of repeat tasks.</t>
+        </is>
+      </c>
+      <c r="I8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Supported migration of workloads from AWS to a new cloud platform.
+\item Assisted with deployment through CI/CD pipelines.
+\item Helped monitor migrated applications.
+\item Supported troubleshooting of migration issues.
+\item Helped automate migration checks.</t>
+        </is>
+      </c>
+      <c r="J8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Assisted in maintaining AWS cloud setups for cloud native products.
+\item Supported CI/CD pipelines and deployment of new releases.
+\item Helped monitor product uptime.
+\item Assisted in troubleshooting production issues.
+\item Supported automation of release steps.</t>
+        </is>
+      </c>
+      <c r="K8" s="30" t="inlineStr">
+        <is>
+          <t>DevOps Engineer I
+\item Supported AWS cloud infrastructure built for high availability.
+\item Assisted in CI/CD pipeline runs and application deployment.
+\item Helped monitor uptime and alerts.
+\item Supported troubleshooting during outages.
+\item Assisted in automating routine checks.</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="30" t="inlineStr">
@@ -6917,6 +7708,106 @@
           <t>UI/UX Designer</t>
         </is>
       </c>
+      <c r="B9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Led UI/UX design for admin and mobile screens, starting from user requirements and wireframes in Figma.
+\item Built clickable prototypes and mock-ups to check flows before hand-off.
+\item Created visual design with consistent typography and color across screens.
+\item Kept every screen within brand guidelines and a shared design system, using responsive web design for web and mobile.
+\item Produced icons and graphics in Adobe Illustrator and Photoshop and eased the web development hand-off, cutting rework by about 20\%.</t>
+        </is>
+      </c>
+      <c r="C9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Designed website layouts and landing pages in Figma, following responsive web design.
+\item Led UI/UX design from requirements to wireframes, prototypes and mock-ups.
+\item Built web graphics, banners and icons in Photoshop and Adobe Illustrator.
+\item Set visual design, typography and color choices that kept pages within brand guidelines and the design system.
+\item Worked with the web development team on hand-off, improving landing-page sign-ups by about 15\%.</t>
+        </is>
+      </c>
+      <c r="D9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Led graphic design of campaign creatives and banners in Photoshop and Adobe Illustrator.
+\item Created UI/UX design for campaign landing screens from client requirements, with wireframes and prototypes in Figma.
+\item Applied visual design, typography and color choices within brand guidelines.
+\item Built a reusable design system for campaign assets, using responsive web design for every screen size.
+\item Eased web development of campaign pages, cutting design turnaround by about 25\%.</t>
+        </is>
+      </c>
+      <c r="E9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Led UI/UX design for web and mobile applications, from requirements to wireframes, prototypes and visual design.
+\item Designed screens in Figma with responsive web design across devices.
+\item Created icons and graphics in Adobe Illustrator and Photoshop.
+\item Kept typography, color and layout consistent with brand guidelines through a shared design system.
+\item Worked with developers on web development hand-off, reducing design-related fixes by about 20\%.</t>
+        </is>
+      </c>
+      <c r="F9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Designed navigation components and graphic elements from gathered user requirements.
+\item Led UI/UX design with wireframes, mock-ups and prototypes in Figma.
+\item Applied visual design, typography and color choices, staying within brand guidelines and the design system.
+\item Produced graphics in Photoshop and Adobe Illustrator and checked responsive web design on all screen sizes.
+\item Worked with the web development team on hand-off, improving task completion in navigation by about 15\%.</t>
+        </is>
+      </c>
+      <c r="G9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Assisted in UI/UX design of admin and mobile screens.
+\item Helped create wireframes in Figma for review.
+\item Supported visual design updates in Photoshop and Adobe Illustrator.
+\item Helped keep screens within brand guidelines.
+\item Checked layouts for responsive web design on web and mobile.</t>
+        </is>
+      </c>
+      <c r="H9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Assisted in UI/UX design of website layouts and landing pages.
+\item Helped create wireframes in Figma.
+\item Supported visual design work in Photoshop and Adobe Illustrator.
+\item Helped keep pages consistent with brand guidelines.
+\item Supported responsive web design for desktop and mobile.</t>
+        </is>
+      </c>
+      <c r="I9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Assisted in UI/UX design of campaign landing screens.
+\item Edited campaign visual design assets in Photoshop and Adobe Illustrator.
+\item Helped create simple wireframes in Figma.
+\item Helped keep creatives within brand guidelines.
+\item Supported responsive web design for campaign pages.</t>
+        </is>
+      </c>
+      <c r="J9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Assisted in UI/UX design for web and mobile applications.
+\item Helped create wireframes in Figma.
+\item Supported visual design work in Photoshop and Adobe Illustrator.
+\item Helped apply brand guidelines across screens.
+\item Checked responsive web design across devices.</t>
+        </is>
+      </c>
+      <c r="K9" s="30" t="inlineStr">
+        <is>
+          <t>UI/UX Designer I
+\item Assisted in UI/UX design of navigation components.
+\item Helped create wireframes in Figma.
+\item Supported visual design in Photoshop and Adobe Illustrator.
+\item Helped keep components within brand guidelines.
+\item Checked responsive web design on different screen sizes.</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="30" t="inlineStr">
@@ -6924,6 +7815,106 @@
           <t>BI / Reporting Developer</t>
         </is>
       </c>
+      <c r="B10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Gathered requirements from business teams and built Power BI dashboards with DAX measures.
+\item Designed data models on a star schema over the data warehouse.
+\item Wrote SQL against source databases and validated data before each refresh.
+\item Cleaned data in MS Excel with pivot tables for one-off reports.
+\item Documented report logic and dashboard usage guides, cutting repeat user questions by about 30\%.</t>
+        </is>
+      </c>
+      <c r="C10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Gathered requirements from business stakeholders and turned them into metrics and reports.
+\item Built interactive Power BI dashboards with DAX and wrote SQL queries across databases.
+\item Developed data models with fact and dimension tables for the data warehouse.
+\item Cleaned and validated data in MS Excel using pivot tables before loading.
+\item Documented data definitions and report logic, reducing report errors by about 20\%.</t>
+        </is>
+      </c>
+      <c r="D10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Built Power BI dashboards and reports with DAX for daily operations.
+\item Gathered dashboard requirements from end users across teams.
+\item Designed data models on a star schema in the data warehouse and wrote SQL against operational databases.
+\item Reviewed, cleaned and validated data in MS Excel with pivot tables.
+\item Wrote documentation for smooth operations and easy maintenance, cutting user requests by about 25\%.</t>
+        </is>
+      </c>
+      <c r="E10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Built Power BI dashboards with DAX for the business systems team.
+\item Designed data models on a star schema for the data warehouse.
+\item Wrote SQL against source databases and validated the loaded data.
+\item Cleaned source data in MS Excel with pivot tables.
+\item Gathered reporting requirements and documented each dashboard, cutting refresh issues by about 20\%.</t>
+        </is>
+      </c>
+      <c r="F10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Built Power BI dashboards and reports with DAX for application users.
+\item Gathered requirements and documented application workflows, user guides and technical setups.
+\item Designed data models with primary and foreign keys on a star schema in the data warehouse.
+\item Wrote SQL against relational databases and validated results.
+\item Cleaned data in MS Excel with pivot tables and formulas, cutting manual report work by about 30\%.</t>
+        </is>
+      </c>
+      <c r="G10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Assisted in building and updating basic dashboards and reports in Power BI for business teams.
+\item Wrote basic SQL queries for report data.
+\item Used MS Excel formulas for one-off reports.
+\item Supported documentation of report logic.
+\item Helped refresh reports on schedule.</t>
+        </is>
+      </c>
+      <c r="H10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Assisted in building interactive Power BI dashboards for business stakeholders.
+\item Wrote basic SQL queries to pull report data.
+\item Prepared supporting reports in MS Excel.
+\item Helped document data definitions.
+\item Supported scheduled report updates.</t>
+        </is>
+      </c>
+      <c r="I10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Assisted in developing Power BI dashboards and reports for daily operations.
+\item Wrote simple SQL queries.
+\item Kept daily trackers in MS Excel.
+\item Supported documentation for smooth operations.
+\item Helped users with report questions.</t>
+        </is>
+      </c>
+      <c r="J10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Assisted in building Power BI dashboards for the business systems team.
+\item Wrote basic SQL queries for dashboard data.
+\item Prepared MS Excel reports for the team.
+\item Helped document each dashboard.
+\item Supported dashboard refreshes.</t>
+        </is>
+      </c>
+      <c r="K10" s="30" t="inlineStr">
+        <is>
+          <t>BI Developer I
+\item Assisted in building basic Power BI dashboards and reports for application users.
+\item Wrote basic SQL queries.
+\item Maintained MS Excel reports.
+\item Supported documentation of application workflows and user guides.
+\item Helped update reports on request.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="30" t="inlineStr">
@@ -6931,6 +7922,106 @@
           <t>Network Engineer</t>
         </is>
       </c>
+      <c r="B11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Led 24/7 network monitoring of routers, switches, firewalls and servers.
+\item Handled incident management, logging incidents in the ITSM ticketing tool and keeping documentation current.
+\item Carried out network troubleshooting of LAN and WAN links, cutting mean time to restore by about 25\%.
+\item Gave technical support on Windows and Linux hosts and handled basic troubleshooting.
+\item Applied network security checks across networking devices and handled installation of new equipment.</t>
+        </is>
+      </c>
+      <c r="C11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Installed, configured and maintained routers, switches and office PCs for office networking.
+\item Led network troubleshooting of LAN, WAN and internet connectivity issues.
+\item Gave technical support to end-users on Windows and Linux, troubleshooting software and access problems.
+\item Set up network monitoring and firewall rules in line with network security practices, cutting outages by about 20\%.
+\item Logged incidents in the ticketing system and documented network configurations and fixes.</t>
+        </is>
+      </c>
+      <c r="D11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Led network monitoring of devices, servers, applications and circuits using enterprise tools.
+\item Ran first-level network troubleshooting with ping, traceroute and port checks across LAN and WAN links.
+\item Checked switch, router and firewall reachability and applied network security fixes.
+\item Managed incidents in the ITSM tool, keeping full documentation for shift handovers, cutting handover gaps by about 30\%.
+\item Gave technical support on Windows and Linux servers and handled installation of new monitoring agents.</t>
+        </is>
+      </c>
+      <c r="E11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Led network troubleshooting of LAN, WAN, Wi-Fi and internet connectivity issues across branches.
+\item Installed and configured routers, switches and firewalls for branch networking.
+\item Set up network monitoring of connectivity and performance, cutting downtime by about 20\%.
+\item Gave technical support to branch users on Windows and Linux systems and logged incidents in the ticketing system.
+\item Maintained network documentation and troubleshooting records, following network security practices.</t>
+        </is>
+      </c>
+      <c r="F11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Resolved customer-reported network issues through tickets in the ITSM system, handling incident management end to end.
+\item Led network troubleshooting across LAN and WAN links, routers and switches.
+\item Configured firewalls and network security settings for customer sites.
+\item Ran network monitoring and installation of network devices on site, cutting repeat tickets by about 25\%.
+\item Gave technical support on Windows and Linux and documented each fix.</t>
+        </is>
+      </c>
+      <c r="G11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Assisted with 24/7 network monitoring of devices.
+\item Supported basic network troubleshooting before handing over to L2.
+\item Helped check router and switch status.
+\item Gave basic technical support to users.
+\item Helped maintain documentation for shift handovers.</t>
+        </is>
+      </c>
+      <c r="H11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Assisted in configuring routers and switches for office networking.
+\item Supported network troubleshooting of connectivity issues.
+\item Helped monitor network performance.
+\item Gave basic technical support to end-users.
+\item Helped document network configurations and troubleshooting steps.</t>
+        </is>
+      </c>
+      <c r="I11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Assisted with network monitoring of devices and circuits.
+\item Supported first-level network troubleshooting with ping and traceroute.
+\item Helped check switch and router reachability.
+\item Supported users with basic technical support.
+\item Helped maintain complete documentation.</t>
+        </is>
+      </c>
+      <c r="J11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Assisted with network troubleshooting of internet connectivity issues at branches.
+\item Supported configuration of routers and switches.
+\item Helped monitor network connectivity and performance.
+\item Gave basic technical support to branch users.
+\item Helped maintain network documentation.</t>
+        </is>
+      </c>
+      <c r="K11" s="30" t="inlineStr">
+        <is>
+          <t>Network Engineer I
+\item Assisted with customer-reported network issues and helped monitor affected links.
+\item Supported network troubleshooting of reported problems.
+\item Helped check routers and switches on site.
+\item Gave basic technical support to customers.
+\item Helped document each fix.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="30" t="inlineStr">
@@ -6938,6 +8029,106 @@
           <t>Field Technician</t>
         </is>
       </c>
+      <c r="B12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Led equipment installation and commissioning of material testing machines at client sites.
+\item Carried out servicing, repair and preventive maintenance, including routine inspection of machines.
+\item Diagnosed mechanical, electrical and electronic faults through on-site troubleshooting, cutting repeat visits by about 20\%.
+\item Handled customer complaints, gave technical support and trained client staff on machine operation.
+\item Kept service records, reports and site documentation accurate, following safety procedures on every visit.</t>
+        </is>
+      </c>
+      <c r="C12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Managed the full ATM lifecycle, from installation and commissioning to servicing and repair.
+\item Scheduled preventive maintenance and inspections to minimise downtime, cutting breakdown calls by about 25\%.
+\item Resolved electrical, electronic and mechanical faults through troubleshooting.
+\item Responded to customer complaints, provided technical support and trained clients on ATM usage.
+\item Maintained service records, reports and documentation, and followed safety standards in the field.</t>
+        </is>
+      </c>
+      <c r="D12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Led installation and commissioning of lithium battery systems, recording commissioning parameters.
+\item Performed preventive maintenance, servicing, repair and scheduled inspection of deployed battery systems.
+\item Diagnosed electrical, electronic and mechanical issues through troubleshooting.
+\item Attended customer complaints, gave first-level technical support and trained customers on operating procedures.
+\item Maintained service reports, installation documentation and commissioning records under safety standards, reducing open complaints by about 20\%.</t>
+        </is>
+      </c>
+      <c r="E12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Handled installation and commissioning of water treatment plant equipment.
+\item Led preventive maintenance, servicing, repair and equipment inspection across sites.
+\item Diagnosed mechanical, electrical and electronic issues in treatment plants through troubleshooting.
+\item Gave technical support to customers, handled complaints and trained operators.
+\item Kept service records, reports and documentation, followed safety protocols, and cut plant downtime by about 15\%.</t>
+        </is>
+      </c>
+      <c r="F12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Performed on-site installation, configuration and commissioning of camera, recorder and GPS products.
+\item Carried out servicing, repair, preventive maintenance and inspection of installed products.
+\item Resolved electrical, electronic and mechanical faults through troubleshooting, cutting repeat visits by about 20\%.
+\item Gave technical support after installation, training customers on daily use and handling complaints.
+\item Kept service reports, records and documentation, following safety standards during field work.</t>
+        </is>
+      </c>
+      <c r="G12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Assisted in installation of material testing machines.
+\item Supported servicing and repair of machines at client sites.
+\item Helped carry out preventive maintenance visits.
+\item Assisted senior engineers in troubleshooting faults.
+\item Gave basic technical support and prepared service reports.</t>
+        </is>
+      </c>
+      <c r="H12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Assisted with ATM installation and setup.
+\item Supported servicing and repair of ATMs.
+\item Helped with scheduled preventive maintenance.
+\item Assisted in troubleshooting ATM malfunctions.
+\item Gave basic technical support and completed service reports.</t>
+        </is>
+      </c>
+      <c r="I12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Assisted with installation of lithium battery systems.
+\item Supported servicing and repair of battery systems.
+\item Helped with preventive maintenance of deployed systems.
+\item Assisted in troubleshooting system faults.
+\item Gave first-level technical support over phone or video and filled in service reports.</t>
+        </is>
+      </c>
+      <c r="J12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Assisted with installation of water treatment plant equipment.
+\item Supported servicing and repair work.
+\item Helped with preventive maintenance at plant sites.
+\item Assisted in troubleshooting plant issues.
+\item Provided basic technical support and prepared service reports.</t>
+        </is>
+      </c>
+      <c r="K12" s="30" t="inlineStr">
+        <is>
+          <t>Field Service Engineer
+\item Assisted with on-site installation of camera and GPS products.
+\item Supported servicing and repair of installed products.
+\item Helped with preventive maintenance visits.
+\item Assisted in troubleshooting product faults.
+\item Gave basic technical support and submitted service reports.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="30" t="inlineStr">
@@ -6945,6 +8136,106 @@
           <t>IT Infra / Support Engineer</t>
         </is>
       </c>
+      <c r="B13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Led first-line IT support on the service desk, logging and resolving requests in the ticketing system.
+\item Resolved Windows, operating system and MS Office issues through troubleshooting and remote support.
+\item Handled desktop support and hardware repairs for laptops, printers and other peripherals.
+\item Installed software, applied patches and updates, and tracked IT assets, cutting repeat issues by about 25\%.
+\item Ran network troubleshooting for networking problems, gave technical support and kept documentation current.</t>
+        </is>
+      </c>
+      <c r="C13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Gave first-level technical support and IT support to office end-users.
+\item Installed, configured and maintained desktops, laptops and printers, including hardware fixes.
+\item Resolved Windows, operating system and MS Office problems on site and through remote support with troubleshooting.
+\item Maintained system updates and patches and kept the IT asset register.
+\item Checked connectivity and networking issues, logged issues in the ticketing system and kept documentation, cutting ticket backlog by about 20\%.</t>
+        </is>
+      </c>
+      <c r="D13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Resolved virtual desktop, networking and access issues through troubleshooting to minimise service disruption.
+\item Gave technical support and IT support to users on Windows and other operating systems.
+\item Handled hardware checks and printer issues for office users.
+\item Installed and patched software, managed IT assets and used remote support tools, cutting downtime by about 20\%.
+\item Ran network troubleshooting, helped MS Office users, and documented fixes in the ITSM ticketing tool.</t>
+        </is>
+      </c>
+      <c r="E13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Provided remote and on-site technical support and IT support to clients.
+\item Handled hardware and software troubleshooting for desktops, laptops, printers and peripherals.
+\item Kept the IT asset and stock register, and installed and patched software for clients.
+\item Resolved Windows, operating system and MS Office issues, and ran network troubleshooting for networking faults.
+\item Logged requests in the ticketing system and kept documentation, cutting resolution time by about 20\%.</t>
+        </is>
+      </c>
+      <c r="F13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Gave L1/L2 technical support and IT support to end users through phone and remote support tools.
+\item Resolved Windows 10/11 operating system and MS Office issues through troubleshooting.
+\item Handled desktop support, hardware faults and printer and peripheral problems.
+\item Installed, updated and patched software applications and tracked IT assets.
+\item Ran network troubleshooting on networking issues, logged every request in the ticketing system and kept documentation, cutting backlog by about 25\%.</t>
+        </is>
+      </c>
+      <c r="G13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Assisted on the IT service desk with incoming IT support requests.
+\item Supported troubleshooting of Windows issues.
+\item Helped with desktop support for staff laptops.
+\item Assisted with network troubleshooting of networking issues.
+\item Documented solutions and gave basic technical support.</t>
+        </is>
+      </c>
+      <c r="H13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Gave first-level technical support to office end-users.
+\item Supported IT support tasks for daily user issues.
+\item Helped with desktop support for desktops and laptops.
+\item Assisted in troubleshooting Windows problems.
+\item Helped with network troubleshooting and kept documentation.</t>
+        </is>
+      </c>
+      <c r="I13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Assisted in troubleshooting desktop and networking issues.
+\item Supported IT support for users on Windows.
+\item Helped with network troubleshooting with the network team.
+\item Gave basic technical support to users.
+\item Helped maintain documentation for knowledge sharing.</t>
+        </is>
+      </c>
+      <c r="J13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Assisted with technical support and IT support for clients.
+\item Supported desktop support for client laptops.
+\item Helped troubleshoot Windows issues.
+\item Assisted with network troubleshooting of networking faults.
+\item Helped document each fix.</t>
+        </is>
+      </c>
+      <c r="K13" s="30" t="inlineStr">
+        <is>
+          <t>IT Support Engineer
+\item Assisted with L1 technical support to end users by phone.
+\item Supported IT support for Windows issues.
+\item Helped with desktop support and troubleshooting.
+\item Assisted with network troubleshooting of networking issues.
+\item Helped keep documentation of solutions.</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="30" t="inlineStr">
@@ -6952,6 +8243,106 @@
           <t>Information Security / SOC Analyst</t>
         </is>
       </c>
+      <c r="B14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Led SIEM alert triage and security monitoring in a playbook-driven SOC.
+\item Investigated incidents through log analysis and EDR data, escalating per runbooks.
+\item Ran vulnerability assessment checks across Linux hosts, networking and cloud security settings.
+\item Used threat intelligence on common attack types to tune alert rules, cutting false positives by about 30\%.
+\item Documented findings, maintained playbooks and wrote reports in line with information security and compliance needs.</t>
+        </is>
+      </c>
+      <c r="C14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Led security monitoring and alert triage on the SIEM, following CERT-In reporting and log-retention rules.
+\item Handled incident response, using EDR and log analysis to confirm scope.
+\item Ran vulnerability assessment on Linux servers, networking devices and cloud workloads, tracking cloud security gaps.
+\item Applied threat intelligence on emerging threats and escalated confirmed cases to senior analysts.
+\item Wrote incident reports and documentation for compliance and information security audits, cutting report turnaround by about 25\%.</t>
+        </is>
+      </c>
+      <c r="D14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Led security and compliance reviews of new and existing third parties.
+\item Ran vulnerability assessment of third-party-facing Linux systems, networking and cloud security settings.
+\item Monitored SIEM and EDR alerts linked to third-party access, with triage and log analysis.
+\item Handled incident response for third-party events and escalated issues to management.
+\item Used threat intelligence and information security standards to write review reports and documentation, cutting review time by about 20\%.</t>
+        </is>
+      </c>
+      <c r="E14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Led security monitoring across endpoint, networking and cloud security tools, triaging SIEM and EDR alerts.
+\item Carried out incident response with log analysis on Linux hosts.
+\item Ran vulnerability assessment and tracked fixes across networking assets.
+\item Applied threat intelligence on common attack types and escalated confirmed threats, cutting response time by about 30\%.
+\item Documented investigations in reports that met information security and compliance needs.</t>
+        </is>
+      </c>
+      <c r="F14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Led security monitoring and SIEM alert triage for the internal IT environment.
+\item Handled incident response using EDR data and log analysis, escalating serious cases.
+\item Ran vulnerability assessment and informed management of security vulnerabilities through regular reports.
+\item Reviewed Linux, networking and cloud security settings against information security and compliance standards.
+\item Used threat intelligence to refresh documentation and playbooks, reducing repeat alerts by about 20\%.</t>
+        </is>
+      </c>
+      <c r="G14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Assisted in monitoring SIEM alerts in a playbook-driven SOC.
+\item Supported first-level alert triage.
+\item Helped investigate incidents as part of incident response.
+\item Supported vulnerability assessment checks.
+\item Documented findings and helped maintain playbooks.</t>
+        </is>
+      </c>
+      <c r="H14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Assisted in SIEM monitoring of security events.
+\item Supported triage of alerts.
+\item Helped with incident response tasks.
+\item Assisted with vulnerability assessment checks.
+\item Helped document investigation findings.</t>
+        </is>
+      </c>
+      <c r="I14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Assisted in monitoring SIEM alerts linked to third-party access.
+\item Supported alert triage for third-party events.
+\item Helped with incident response on third-party issues.
+\item Supported vulnerability assessment of third-party systems.
+\item Helped document review findings.</t>
+        </is>
+      </c>
+      <c r="J14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Assisted in monitoring SIEM alerts across security tools.
+\item Supported alert triage.
+\item Helped with incident response under senior guidance.
+\item Assisted in vulnerability assessment tasks.
+\item Helped document each investigation.</t>
+        </is>
+      </c>
+      <c r="K14" s="30" t="inlineStr">
+        <is>
+          <t>SOC Analyst I
+\item Assisted in SIEM monitoring for the internal IT environment.
+\item Supported first-level triage of alerts.
+\item Helped with incident response steps.
+\item Supported vulnerability assessment and basic security hygiene checks.
+\item Helped document findings for the team.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="30" t="inlineStr">
@@ -6959,11 +8350,211 @@
           <t>ERP Consultant</t>
         </is>
       </c>
+      <c r="B15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Gathered client requirements and mapped business processes before configuring and customising the client's ERP system and business apps.
+\item Led implementation and testing of configured solutions, including UAT with client users.
+\item Set up integration between the client's business apps and SAP for smooth data flow.
+\item Trained end users, gave technical support and resolved issues through troubleshooting, cutting open issues by about 25\%.
+\item Prepared documentation and reports in MS Excel, maintained master data and worked with clients in English.</t>
+        </is>
+      </c>
+      <c r="C15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Mapped purchasing, warehouse and order-management business processes into the ERP system, with SAP as the base.
+\item Gathered requirements and wrote clear workflows and acceptance criteria.
+\item Configured modules and led implementation, testing and UAT.
+\item Investigated ERP data issues through troubleshooting, gave technical support and trained users, reducing process errors by about 20\%.
+\item Maintained master data, built integrations and reports, and wrote documentation in English using MS Excel.</t>
+        </is>
+      </c>
+      <c r="D15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Implemented and configured ERP solutions for clients, including SAP modules.
+\item Studied business requirements and mapped business processes into the system.
+\item Led testing and UAT, then trained end-users on new processes.
+\item Resolved technical issues through troubleshooting and technical support, cutting go-live issues by about 25\%.
+\item Managed master data, integration with other systems, reports and documentation, working in English and MS Excel.</t>
+        </is>
+      </c>
+      <c r="E15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Reviewed customer requirements and mapped business processes into the ERP system, with SAP exposure.
+\item Configured modules and handled implementation for each customer.
+\item Coached customers through individual training sessions and gave technical support.
+\item Ran testing and UAT and resolved issues through troubleshooting, improving onboarding time by about 20\%.
+\item Prepared documentation and reports, set up master data and integration, in English and MS Excel.</t>
+        </is>
+      </c>
+      <c r="F15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Led ERP implementation tasks on SAP, including configuration and integration activities.
+\item Gathered client requirements and mapped business processes.
+\item Ran testing and UAT, and checked master data before go-live.
+\item Handled client issue troubleshooting and technical support, and trained users, cutting repeat issues by about 30\%.
+\item Maintained test cases, issue reports and implementation documentation in English, using MS Excel.</t>
+        </is>
+      </c>
+      <c r="G15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Assisted in ERP implementation for clients.
+\item Helped gather client requirements.
+\item Supported testing of new solutions.
+\item Helped train end users.
+\item Prepared basic documentation and user notes.</t>
+        </is>
+      </c>
+      <c r="H15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Assisted with ERP implementation for supply chain teams.
+\item Helped capture user requirements.
+\item Supported testing of new workflows.
+\item Helped train users on new screens.
+\item Supported documentation of workflows.</t>
+        </is>
+      </c>
+      <c r="I15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Assisted in ERP implementation projects for clients.
+\item Helped document business requirements.
+\item Supported testing of new solutions.
+\item Helped train end-users on new systems.
+\item Prepared user manuals and documentation.</t>
+        </is>
+      </c>
+      <c r="J15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Assisted with ERP implementation for new customers.
+\item Helped note customer requirements.
+\item Supported testing during onboarding.
+\item Helped run training sessions for customers.
+\item Helped maintain onboarding documentation.</t>
+        </is>
+      </c>
+      <c r="K15" s="30" t="inlineStr">
+        <is>
+          <t>ERP Consultant I
+\item Supported ERP implementation tasks.
+\item Helped gather client requirements.
+\item Assisted with testing activities.
+\item Helped train users.
+\item Maintained implementation documentation.</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="30" t="inlineStr">
         <is>
           <t>SAP Technical Consultant</t>
+        </is>
+      </c>
+      <c r="B16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Built ABAP programs and reports on SAP S/4HANA for purchasing and plant processes.
+\item Gathered requirements from functional designs and turned them into technical specifications with clear documentation.
+\item Configured SAP MM settings for purchasing during implementation of new features.
+\item Led testing, debugging and troubleshooting of custom objects, cutting defect turnaround by about 25\%.
+\item Worked on database operations and the technical architecture, and gave technical support to business users.</t>
+        </is>
+      </c>
+      <c r="C16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Delivered ABAP enhancements for the SAP Plant Maintenance module on S/4HANA.
+\item Led implementation and support tasks with the IT team, including module configuration.
+\item Gathered requirements from maintenance users and prepared documentation and status reports.
+\item Handled testing, debugging and troubleshooting of maintenance programs, reducing open issues by about 20\%.
+\item Worked with SAP MM touchpoints, database tables and the technical architecture, and gave technical support to users.</t>
+        </is>
+      </c>
+      <c r="D16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Built ABAP reports on SAP S/4HANA for HR module projects.
+\item Gathered business requirements for personnel administration and wrote functional documentation and user manuals.
+\item Performed SAP configuration during implementation and support projects.
+\item Led testing, debugging and troubleshooting of custom objects, cutting rework by about 20\%.
+\item Handled database operations and technical architecture checks, gave end-user technical support, and covered SAP MM touchpoints.</t>
+        </is>
+      </c>
+      <c r="E16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Delivered end-to-end implementation, rollout and support of SAP S/4HANA projects.
+\item Built ABAP programs and reports from functional requirements, with technical documentation.
+\item Configured SAP MM settings for rollout sites.
+\item Led testing, debugging and troubleshooting during rollout, cutting post-go-live issues by about 30\%.
+\item Gave technical support to users and worked on database operations and the solution architecture.</t>
+        </is>
+      </c>
+      <c r="F16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Built ABAP programs and reports for make-to-stock and make-to-order scenarios on SAP S/4HANA.
+\item Ran end-to-end scenario testing of each flow, plus debugging and troubleshooting.
+\item Set up master configuration for SAP MM materials.
+\item Gathered requirements and wrote documentation and test reports during implementation.
+\item Gave technical support on database and architecture questions, reducing open issues by about 20\%.</t>
+        </is>
+      </c>
+      <c r="G16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Assisted in developing ABAP programs on SAP S/4HANA for plant processes.
+\item Supported basic SAP configuration under senior guidance.
+\item Helped with testing of custom objects.
+\item Assisted in troubleshooting technical issues.
+\item Supported preparation of technical documentation.</t>
+        </is>
+      </c>
+      <c r="H16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Assisted in ABAP changes for the SAP Plant Maintenance module on S/4HANA.
+\item Supported module configuration tasks.
+\item Helped with testing of maintenance programs.
+\item Assisted in troubleshooting user issues.
+\item Helped maintain documentation.</t>
+        </is>
+      </c>
+      <c r="I16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Assisted in ABAP development on SAP S/4HANA for HR projects.
+\item Performed basic SAP configuration under senior consultant guidance.
+\item Helped with testing of changes.
+\item Assisted in troubleshooting issues.
+\item Supported functional documentation and user manuals.</t>
+        </is>
+      </c>
+      <c r="J16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Assisted in ABAP development during SAP S/4HANA rollout projects.
+\item Supported configuration tasks for rollout sites.
+\item Helped with testing during rollout.
+\item Assisted in troubleshooting rollout issues.
+\item Helped maintain project documentation.</t>
+        </is>
+      </c>
+      <c r="K16" s="30" t="inlineStr">
+        <is>
+          <t>SAP ABAP Consultant I
+\item Assisted in ABAP development for make-to-stock and make-to-order scenarios on SAP S/4HANA.
+\item Supported master configuration tasks.
+\item Helped with end-to-end scenario testing.
+\item Assisted in troubleshooting scenario issues.
+\item Supported documentation of test results.</t>
         </is>
       </c>
     </row>
@@ -7026,51 +8617,51 @@
       <c r="G17" s="30" t="inlineStr">
         <is>
           <t>Warehouse Executive
-\item Supported day-to-day operations management and warehouse operations at a shipment hub.
-\item Assisted with inbound and outbound shipment handling as part of daily logistics operations.
-\item Helped with inventory management by flagging shipment discrepancies and damages.
-\item Supported timely updating of operational records and compliance with company policies.
-\item Assisted in preparing daily operational reports for the reporting manager.</t>
+\item Assisted with inbound receiving of shipments at a shipment hub.
+\item Supported outbound dispatch of shipments.
+\item Helped with inventory management and daily stock checks.
+\item Supported timely updating of records in compliance with company policies.
+\item Assisted in preparing daily reports for the reporting manager.</t>
         </is>
       </c>
       <c r="H17" s="30" t="inlineStr">
         <is>
           <t>Warehouse Executive
-\item Supported warehouse operations and operations management at a distribution warehouse.
-\item Assisted with inbound receipt and outbound dispatch of goods as part of daily logistics operations.
-\item Helped with inventory management and reported quantity discrepancies and damaged goods.
-\item Supported accurate record keeping for incoming and outgoing goods, in compliance with company policies.
-\item Assisted in preparing inventory-related reports as required.</t>
+\item Assisted with inbound receipt of goods at a distribution warehouse.
+\item Supported outbound dispatch and distribution of goods.
+\item Helped with inventory management of stored goods.
+\item Supported accurate record keeping in compliance with company policies.
+\item Assisted in preparing inventory-related reports.</t>
         </is>
       </c>
       <c r="I17" s="30" t="inlineStr">
         <is>
           <t>Dispatch Executive
-\item Supported warehouse operations and operations management for finished goods at a manufacturing yard.
-\item Assisted with inward receipts and outbound dispatch as part of finished-goods logistics operations.
-\item Helped with inventory management of finished goods in the yard and reported dispatch delays and damaged goods.
-\item Supported daily dispatch logs and stock record keeping in line with logistics compliance.
+\item Assisted with inward receipts of finished goods at a manufacturing yard.
+\item Supported outbound dispatch of finished goods.
+\item Helped with inventory management of goods in the yard.
+\item Supported daily dispatch logs and stock records in line with logistics compliance.
+\item Assisted in preparing day-to-day reports.</t>
+        </is>
+      </c>
+      <c r="J17" s="30" t="inlineStr">
+        <is>
+          <t>Inventory Executive
+\item Assisted with inbound receiving of goods for a hotel.
+\item Supported outbound dispatch of stock to hotel departments.
+\item Helped with inventory management and stock counts.
+\item Supported accurate record keeping in compliance with company policies.
+\item Assisted with month-end inventory reports.</t>
+        </is>
+      </c>
+      <c r="K17" s="30" t="inlineStr">
+        <is>
+          <t>Store Officer
+\item Assisted with inward receipt of material in a production environment.
+\item Supported outbound dispatch of material to depots.
+\item Helped with inventory management of material stocks.
+\item Supported accurate stock records in compliance with company policies and regulatory requirements.
 \item Assisted in preparing day-to-day operational reports.</t>
-        </is>
-      </c>
-      <c r="J17" s="30" t="inlineStr">
-        <is>
-          <t>Inventory Executive
-\item Supported warehouse operations and operations management for a hotel's stock.
-\item Assisted with inbound receiving of goods and outbound dispatch as part of daily logistics operations.
-\item Helped with inventory management and reported damaged items and stock discrepancies.
-\item Supported accurate record keeping for stock movements, in compliance with company policies.
-\item Assisted with month-end inventory reports as required.</t>
-        </is>
-      </c>
-      <c r="K17" s="30" t="inlineStr">
-        <is>
-          <t>Store Officer
-\item Supported warehouse operations and operations management in a production environment.
-\item Assisted with inward receipt of material and outbound dispatch to depots as part of logistics operations.
-\item Helped with inventory management and reported damaged goods, missing items and excess stock.
-\item Supported accurate record keeping of stock movements, in compliance with company policies and regulatory requirements.
-\item Assisted in preparing day-to-day operational reports for circulation.</t>
         </is>
       </c>
     </row>
@@ -7080,6 +8671,106 @@
           <t>HR / Talent Acquisition Specialist</t>
         </is>
       </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Led end-to-end recruitment and bulk hiring for blue-collar non-IT roles, from requirement gathering with operations managers to joining.
+\item Sourced candidates through Naukri, job portals, referrals and walk-in drives, building a steady talent pipeline.
+\item Screened resumes and conducted initial telephonic interviews, then coordinated interviews with operations managers.
+\item Handled salary negotiation and onboarding, cutting offer dropouts by about 20\%.
+\item Kept recruitment trackers and MIS up to date, shared hiring reports, spoke with candidates in English and covered engineering hiring when needed.</t>
+        </is>
+      </c>
+      <c r="C18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Led end-to-end bulk recruitment for telecalling, telesales and telecollection non-IT roles.
+\item Sourced through Naukri and other job portals and built a candidate pipeline for high-volume hiring requirements.
+\item Screened candidates, conducted telephonic interviews in English and coordinated interviews with hiring managers.
+\item Handled offers and salary discussions and drove onboarding until joining, raising joining rates by about 25\%.
+\item Maintained recruitment trackers, daily hiring reports and pipeline updates, and covered engineering hiring when needed.</t>
+        </is>
+      </c>
+      <c r="D18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Led end-to-end recruitment for BPO, BPS and ITES roles, working from job descriptions and requirements.
+\item Sourced candidates on Naukri and LinkedIn and kept a pipeline for open positions.
+\item Screened candidates on skills, experience and location, conducted interviews and coordinated interviews with clients.
+\item Ran bulk hiring drives for non-IT and technical roles, and negotiated salary before onboarding.
+\item Maintained the recruitment MIS, shared reports and spoke with candidates in English, cutting time-to-close by about 20\%.</t>
+        </is>
+      </c>
+      <c r="E18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Led end-to-end recruitment and bulk hiring for field sales and other non-IT roles.
+\item Sourced through Naukri, LinkedIn and job portals to build a pipeline for hiring targets.
+\item Screened resumes, conducted telephonic interviews, and coordinated interviews with sales managers.
+\item Gathered manpower requirements, negotiated salary and managed onboarding, cutting no-shows by about 20\%.
+\item Kept recruitment trackers and daily reports, worked with candidates in English, and covered engineering hiring when needed.</t>
+        </is>
+      </c>
+      <c r="F18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Led end-to-end recruitment for engineering and professional roles, plus bulk hiring for non-IT support roles.
+\item Sourced candidates through LinkedIn, Naukri and job portals, keeping a pipeline of suitable profiles.
+\item Gathered requirements from hiring managers, screened resumes and conducted interviews in English.
+\item Coordinated interviews, negotiated salary and released offer letters, then handled onboarding.
+\item Maintained recruitment trackers and MIS and shared weekly reports, reducing time-to-hire by about 20\%.</t>
+        </is>
+      </c>
+      <c r="G18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Assisted with end-to-end recruitment for blue-collar roles.
+\item Helped source candidates through Naukri and job portals.
+\item Supported resume screening and initial candidate calls.
+\item Helped schedule interviews with operations managers.
+\item Updated recruitment trackers daily.</t>
+        </is>
+      </c>
+      <c r="H18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Supported end-to-end recruitment for telecalling and telesales roles.
+\item Helped source candidates on Naukri and other job portals.
+\item Assisted with screening of candidates.
+\item Helped coordinate interviews with hiring managers.
+\item Maintained recruitment trackers.</t>
+        </is>
+      </c>
+      <c r="I18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Assisted with end-to-end recruitment for BPO and ITES roles.
+\item Helped source candidates on Naukri and LinkedIn.
+\item Supported screening of candidates against job descriptions.
+\item Helped schedule interviews with clients.
+\item Updated candidate details in the recruitment MIS.</t>
+        </is>
+      </c>
+      <c r="J18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Assisted with end-to-end recruitment for field sales roles.
+\item Helped source candidates through job portals.
+\item Supported resume screening.
+\item Helped coordinate interviews with sales managers.
+\item Kept recruitment trackers up to date.</t>
+        </is>
+      </c>
+      <c r="K18" s="30" t="inlineStr">
+        <is>
+          <t>HR Recruiter
+\item Supported end-to-end recruitment for professional roles.
+\item Helped source candidates on LinkedIn and Naukri.
+\item Assisted with resume screening.
+\item Helped schedule interviews with hiring managers.
+\item Maintained recruitment trackers and MIS entries.</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="30" t="inlineStr">
@@ -7087,11 +8778,211 @@
           <t>Finance and Accounts Executive</t>
         </is>
       </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Ran accounts payable for supplier invoices and billing across locations, working with vendors to clear open items.
+\item Maintained ledgers in Tally and MS Excel, handling bookkeeping and accounting entries.
+\item Led bank and vendor reconciliation and tracked accounts receivable ageing, cutting unreconciled items by about 30\%.
+\item Prepared month-end closing reports and audit schedules for cash checks across locations.
+\item Kept records and documentation in the ERP system in line with compliance rules.</t>
+        </is>
+      </c>
+      <c r="C19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Handled accounting operations, bookkeeping and ledger entries in Tally and the ERP system.
+\item Verified invoices for accuracy and compliance, and created new vendor profiles.
+\item Led reconciliation of accounts payable and accounts receivable balances.
+\item Filed documentation and kept records in the document management system, reducing missing papers by about 25\%.
+\item Prepared ageing reports and month-end closing schedules in MS Excel and handled audit requests.</t>
+        </is>
+      </c>
+      <c r="D19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Raised customer invoices and billing for client contracts and tracked accounts receivable ageing.
+\item Reconciled sales entries, invoices and customer ledgers in Tally and MS Excel.
+\item Led month-end closing for billing and revenue and handled audit requests, cutting close time by about 20\%.
+\item Handled accounts payable for vendors on new invoicing and ERP systems.
+\item Maintained customer agreements, records and documentation in line with compliance, and prepared accounting reports.</t>
+        </is>
+      </c>
+      <c r="E19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Verified receipts and expense categories for policy compliance before payment.
+\item Processed accounts payable invoices with vendors and approvers.
+\item Led reconciliation of employee and vendor accounts in Tally and MS Excel, with accounts receivable checks.
+\item Prepared month-end closing entries, reports and audit requests, reducing claim errors by about 20\%.
+\item Kept bookkeeping records and documentation in the ERP system and ensured accounting accuracy.</t>
+        </is>
+      </c>
+      <c r="F19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Ran accounts payable and accounts receivable operations, including invoice processing and billing.
+\item Recorded AP and AR invoices in the ERP system and kept bookkeeping in Tally.
+\item Led vendor, bank and customer reconciliation in MS Excel, cutting reconciliation backlog by about 25\%.
+\item Prepared month-end closing entries and accounting reports and handled audit requests.
+\item Maintained accurate financial records and documentation in line with compliance rules.</t>
+        </is>
+      </c>
+      <c r="G19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Assisted with invoice processing and billing across locations.
+\item Supported accounting entries in Tally.
+\item Helped with bank reconciliation.
+\item Maintained records in MS Excel.
+\item Helped prepare MS Office summaries for the accounts team.</t>
+        </is>
+      </c>
+      <c r="H19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Assisted with accounting operations in Tally.
+\item Helped verify invoices for accuracy.
+\item Supported reconciliation of accounts.
+\item Filed and maintained accounting records.
+\item Used MS Excel and MS Word for daily work.</t>
+        </is>
+      </c>
+      <c r="I19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Assisted in raising customer invoices and billing.
+\item Helped reconcile sales entries and invoices.
+\item Supported accounting entries in Tally.
+\item Maintained billing records.
+\item Used MS Excel for billing trackers.</t>
+        </is>
+      </c>
+      <c r="J19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Assisted in checking expense invoices.
+\item Supported reconciliation of employee accounts.
+\item Helped post accounting entries in Tally.
+\item Maintained claim records in MS Excel.
+\item Helped keep receipts and records in order.</t>
+        </is>
+      </c>
+      <c r="K19" s="30" t="inlineStr">
+        <is>
+          <t>Accounts Executive
+\item Assisted with invoice processing and billing.
+\item Helped record accounting entries in Tally.
+\item Supported account reconciliation.
+\item Maintained accurate records.
+\item Used MS Excel for daily trackers.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="30" t="inlineStr">
         <is>
           <t>Customer Support Associate</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Handled customer queries through email and live chat, plus inbound calls, in clear written and spoken English.
+\item Used product knowledge to answer feature and service questions and resolved simple technical issues through troubleshooting.
+\item Used computer systems to log every interaction in the CRM and ticketing tool with accurate data entry and records.
+\item Followed SOPs and escalated complex issues to the right team.
+\item Met productivity and CSAT targets, raising customer satisfaction scores by about 10\%.</t>
+        </is>
+      </c>
+      <c r="C20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Handled inbound calls and enquiries from parents, students and school staff across admissions and general questions.
+\item Answered further queries by email and chat in clear English, using product knowledge of admissions services.
+\item Gave basic troubleshooting by phone and escalated complex issues to engineering.
+\item Logged each interaction in the CRM and ticketing system on the computer, with accurate data entry and records.
+\item Followed SOPs and met CSAT targets, cutting repeat calls by about 15\%.</t>
+        </is>
+      </c>
+      <c r="D20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Answered service, product and technical questions on software features through calls, email and chat.
+\item Resolved simple software issues through troubleshooting, using product knowledge and standard protocols.
+\item Logged cases in the ticketing system and CRM on computer systems, with accurate data entry and records.
+\item Escalated complex cases and kept English replies clear and accurate.
+\item Met productivity targets, improving CSAT by about 10\%.</t>
+        </is>
+      </c>
+      <c r="E20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Handled inbound and outbound customer calls and resolved customer queries in English.
+\item Gave accurate product information and resolved basic issues through troubleshooting.
+\item Updated call details in the CRM and ticketing system with accurate data entry and records, using computer systems daily.
+\item Followed company policies and SOPs and escalated unresolved issues to the concerned department.
+\item Covered email and chat support during peak hours and met AHT and CSAT targets, cutting handling time by about 15\%.</t>
+        </is>
+      </c>
+      <c r="F20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Handled partner queries on incentive eligibility, payments and payouts through calls, email and chat.
+\item Used product knowledge of incentive schemes and troubleshooting to resolve issues quickly.
+\item Logged each case in the ticketing system and CRM on the computer with accurate data entry and records.
+\item Followed SOPs and escalated complex cases to the concerned team.
+\item Met CSAT targets in clear written English, cutting turnaround time by about 20\%.</t>
+        </is>
+      </c>
+      <c r="G20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Assisted customers with written queries in clear English.
+\item Supported phone calls when inbound volume was high.
+\item Helped answer product questions using product knowledge.
+\item Kept records of customer interactions on the computer.
+\item Followed SOPs and escalated complex issues to the right team.</t>
+        </is>
+      </c>
+      <c r="H20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Assisted with inbound calls and enquiries from parents and students.
+\item Helped answer admissions questions using product knowledge.
+\item Supported spoken and written English replies.
+\item Kept accurate records on the computer.
+\item Followed SOPs and escalated complex issues to senior staff.</t>
+        </is>
+      </c>
+      <c r="I20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Assisted with inbound calls on product and service questions.
+\item Supported customers using product knowledge of software features.
+\item Kept records of each interaction on the computer.
+\item Followed standard protocols and escalated complex issues.
+\item Helped write clear English replies to queries.</t>
+        </is>
+      </c>
+      <c r="J20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Assisted with inbound and outbound customer calls.
+\item Helped resolve customer queries in English.
+\item Shared product knowledge on services and processes.
+\item Updated call records on the computer.
+\item Followed company policies and SOPs and escalated unresolved issues.</t>
+        </is>
+      </c>
+      <c r="K20" s="30" t="inlineStr">
+        <is>
+          <t>Customer Support Associate
+\item Assisted partners with incentive queries over phone calls.
+\item Helped explain incentive schemes using product knowledge.
+\item Kept records of each query on the computer.
+\item Followed SOPs and escalated complex cases.
+\item Wrote clear English replies to partners.</t>
         </is>
       </c>
     </row>

</xml_diff>